<commit_message>
improved case study 2
</commit_message>
<xml_diff>
--- a/python/CaseStudy_2/outputs/results/CaseStudy_2_results.xlsx
+++ b/python/CaseStudy_2/outputs/results/CaseStudy_2_results.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Descriptives" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clusters" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baseline model" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Band breakdown" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -864,4 +865,200 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Band</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Freq min (Hz)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Freq max (Hz)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Cluster mass</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>N points</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>p_raw</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>p_bonferroni (x5)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Significant (p&lt;0.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>delta</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-494.2905727731217</v>
+      </c>
+      <c r="E2" t="n">
+        <v>221</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>theta</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-1963.327834746321</v>
+      </c>
+      <c r="E3" t="n">
+        <v>827</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>alpha</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-897.2865649535978</v>
+      </c>
+      <c r="E4" t="n">
+        <v>393</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.4299999999999999</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>beta</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" t="n">
+        <v>30</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-3378.161141946385</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1421</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>gamma</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>30</v>
+      </c>
+      <c r="C6" t="n">
+        <v>40</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-1043.985071773055</v>
+      </c>
+      <c r="E6" t="n">
+        <v>444</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
CS2 with missign data
</commit_message>
<xml_diff>
--- a/python/CaseStudy_2/outputs/results/CaseStudy_2_results.xlsx
+++ b/python/CaseStudy_2/outputs/results/CaseStudy_2_results.xlsx
@@ -452,12 +452,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>65.38 ± 8.27</t>
+          <t>65.30 ± 6.63</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>[45.00, 86.00]</t>
+          <t>[49.00, 82.00]</t>
         </is>
       </c>
     </row>
@@ -492,12 +492,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>96.02 ± 11.34</t>
+          <t>96.10 ± 11.15</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>[73.50, 120.10]</t>
+          <t>[74.00, 119.00]</t>
         </is>
       </c>
     </row>
@@ -512,12 +512,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>21.63 ± 6.10</t>
+          <t>21.73 ± 6.00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>[8.17, 30.00]</t>
+          <t>[8.00, 30.00]</t>
         </is>
       </c>
     </row>
@@ -587,22 +587,22 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>-4620.506215346426</v>
+        <v>-4059.667541570288</v>
       </c>
       <c r="D2" t="n">
-        <v>1954</v>
+        <v>1719</v>
       </c>
       <c r="E2" t="n">
-        <v>15.869140625</v>
+        <v>16.11328125</v>
       </c>
       <c r="F2" t="n">
-        <v>39.794921875</v>
+        <v>39.55078125</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8597051013585675</v>
+        <v>0.8620512906406709</v>
       </c>
       <c r="H2" t="n">
-        <v>0.194</v>
+        <v>0.196</v>
       </c>
     </row>
     <row r="3">
@@ -615,22 +615,22 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>-3512.153969299777</v>
+        <v>-3343.064403478603</v>
       </c>
       <c r="D3" t="n">
-        <v>1514</v>
+        <v>1442</v>
       </c>
       <c r="E3" t="n">
         <v>1.220703125</v>
       </c>
       <c r="F3" t="n">
-        <v>15.380859375</v>
+        <v>14.16015625</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8868445889033146</v>
+        <v>0.8841820310696296</v>
       </c>
       <c r="H3" t="n">
-        <v>0.234</v>
+        <v>0.224</v>
       </c>
     </row>
     <row r="4">
@@ -643,10 +643,10 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>-20.91130961324618</v>
+        <v>-18.61123439676801</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E4" t="n">
         <v>14.6484375</v>
@@ -658,7 +658,7 @@
         <v>0.9788428578997501</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7695</v>
+        <v>0.786</v>
       </c>
     </row>
     <row r="5">
@@ -671,22 +671,22 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>-15.19358365984864</v>
+        <v>-12.84195091156641</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E5" t="n">
-        <v>28.076171875</v>
+        <v>33.935546875</v>
       </c>
       <c r="F5" t="n">
-        <v>29.541015625</v>
+        <v>34.423828125</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9693068314986495</v>
+        <v>0.5706174287489987</v>
       </c>
       <c r="H5" t="n">
-        <v>0.791</v>
+        <v>0.8095</v>
       </c>
     </row>
     <row r="6">
@@ -699,22 +699,22 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>-10.5445090885832</v>
+        <v>-8.624364012887176</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>19.287109375</v>
+        <v>28.076171875</v>
       </c>
       <c r="F6" t="n">
-        <v>19.775390625</v>
+        <v>28.80859375</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8711540506952616</v>
+        <v>0.9693068314986495</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.835</v>
       </c>
     </row>
     <row r="7">
@@ -727,10 +727,10 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>-2457.618407519443</v>
+        <v>-2432.35014499723</v>
       </c>
       <c r="D7" t="n">
-        <v>1048</v>
+        <v>1038</v>
       </c>
       <c r="E7" t="n">
         <v>1.220703125</v>
@@ -739,10 +739,10 @@
         <v>7.8125</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9110688350528854</v>
+        <v>0.9086030020715889</v>
       </c>
       <c r="H7" t="n">
-        <v>0.039</v>
+        <v>0.0375</v>
       </c>
     </row>
   </sheetData>
@@ -793,16 +793,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29.78358027501667</v>
+        <v>31.66976986875707</v>
       </c>
       <c r="C2" t="n">
-        <v>15.15696405366375</v>
+        <v>14.66843094952766</v>
       </c>
       <c r="D2" t="n">
-        <v>0.05716627778586626</v>
+        <v>0.03758745612161177</v>
       </c>
       <c r="E2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -812,13 +812,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-0.3163781083269208</v>
+        <v>-0.3329664907929477</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5717889072205569</v>
+        <v>0.5710290328456656</v>
       </c>
       <c r="D3" t="n">
-        <v>0.583469479592632</v>
+        <v>0.5634618272830111</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -831,13 +831,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-0.178927089426051</v>
+        <v>-0.2006594618900564</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1183309325003061</v>
+        <v>0.1461265368783622</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1392405311190506</v>
+        <v>0.1781862784956756</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -850,13 +850,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.07756440996850156</v>
+        <v>0.07558691998685743</v>
       </c>
       <c r="C5" t="n">
-        <v>0.08982284277303311</v>
+        <v>0.0895276682326293</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3935649792430459</v>
+        <v>0.4040856564101106</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -931,16 +931,16 @@
         <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>-494.2905727731217</v>
+        <v>-544.6823506512508</v>
       </c>
       <c r="E2" t="n">
-        <v>221</v>
+        <v>242</v>
       </c>
       <c r="F2" t="n">
-        <v>0.076</v>
+        <v>0.073</v>
       </c>
       <c r="G2" t="n">
-        <v>0.38</v>
+        <v>0.365</v>
       </c>
       <c r="H2" t="b">
         <v>0</v>
@@ -959,16 +959,16 @@
         <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>-1963.327834746321</v>
+        <v>-1887.667794345979</v>
       </c>
       <c r="E3" t="n">
-        <v>827</v>
+        <v>796</v>
       </c>
       <c r="F3" t="n">
-        <v>0.027</v>
+        <v>0.023</v>
       </c>
       <c r="G3" t="n">
-        <v>0.135</v>
+        <v>0.115</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -987,16 +987,16 @@
         <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>-897.2865649535978</v>
+        <v>-761.193300977685</v>
       </c>
       <c r="E4" t="n">
-        <v>393</v>
+        <v>335</v>
       </c>
       <c r="F4" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.0795</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4299999999999999</v>
+        <v>0.3975</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -1015,16 +1015,16 @@
         <v>30</v>
       </c>
       <c r="D5" t="n">
-        <v>-3378.161141946385</v>
+        <v>-3002.994657672818</v>
       </c>
       <c r="E5" t="n">
-        <v>1421</v>
+        <v>1263</v>
       </c>
       <c r="F5" t="n">
-        <v>0.075</v>
+        <v>0.0665</v>
       </c>
       <c r="G5" t="n">
-        <v>0.375</v>
+        <v>0.3325</v>
       </c>
       <c r="H5" t="b">
         <v>0</v>
@@ -1043,16 +1043,16 @@
         <v>40</v>
       </c>
       <c r="D6" t="n">
-        <v>-1043.985071773055</v>
+        <v>-877.7029385932183</v>
       </c>
       <c r="E6" t="n">
-        <v>444</v>
+        <v>376</v>
       </c>
       <c r="F6" t="n">
-        <v>0.123</v>
+        <v>0.1315</v>
       </c>
       <c r="G6" t="n">
-        <v>0.615</v>
+        <v>0.6575</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>

</xml_diff>